<commit_message>
chore(data): 同步 2026-09-19（共 207 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$206</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$209</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E206"/>
+  <dimension ref="A1:E209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1741,21 +1741,21 @@
         <v>53</v>
       </c>
       <c r="B55" s="4" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Bisu</t>
         </is>
       </c>
     </row>
@@ -1764,21 +1764,21 @@
         <v>54</v>
       </c>
       <c r="B56" s="8" t="n">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Bisu</t>
         </is>
       </c>
     </row>
@@ -1787,7 +1787,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="4" t="n">
-        <v>46113</v>
+        <v>46111</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="8" t="n">
-        <v>46114</v>
+        <v>46112</v>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
@@ -1819,12 +1819,12 @@
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -1833,16 +1833,16 @@
         <v>57</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>46115</v>
+        <v>46113</v>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>2:4</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -1856,21 +1856,21 @@
         <v>58</v>
       </c>
       <c r="B60" s="8" t="n">
-        <v>46116</v>
+        <v>46114</v>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>0:4</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -1879,21 +1879,21 @@
         <v>59</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>46118</v>
+        <v>46115</v>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Mong</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -1902,21 +1902,21 @@
         <v>60</v>
       </c>
       <c r="B62" s="8" t="n">
-        <v>46119</v>
+        <v>46116</v>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>0:4</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Action</t>
         </is>
       </c>
     </row>
@@ -1925,11 +1925,11 @@
         <v>61</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>46120</v>
+        <v>46118</v>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Mong</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Stork</t>
         </is>
       </c>
     </row>
@@ -1948,21 +1948,21 @@
         <v>62</v>
       </c>
       <c r="B64" s="8" t="n">
-        <v>46120</v>
+        <v>46119</v>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Sorry</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -1971,21 +1971,21 @@
         <v>63</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>46121</v>
+        <v>46120</v>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -1994,21 +1994,21 @@
         <v>64</v>
       </c>
       <c r="B66" s="8" t="n">
-        <v>46122</v>
+        <v>46120</v>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -2017,21 +2017,21 @@
         <v>65</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>46123</v>
+        <v>46121</v>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Rush</t>
         </is>
       </c>
     </row>
@@ -2040,21 +2040,21 @@
         <v>66</v>
       </c>
       <c r="B68" s="8" t="n">
-        <v>46123</v>
+        <v>46122</v>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Sharp</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -2063,21 +2063,21 @@
         <v>67</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>46124</v>
+        <v>46123</v>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Bisu</t>
         </is>
       </c>
     </row>
@@ -2086,21 +2086,21 @@
         <v>68</v>
       </c>
       <c r="B70" s="8" t="n">
-        <v>46125</v>
+        <v>46123</v>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Mong</t>
+          <t>Bisu</t>
         </is>
       </c>
     </row>
@@ -2109,21 +2109,21 @@
         <v>69</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>46126</v>
+        <v>46124</v>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -2132,21 +2132,21 @@
         <v>70</v>
       </c>
       <c r="B72" s="8" t="n">
-        <v>46127</v>
+        <v>46125</v>
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>1:4</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>Mong</t>
         </is>
       </c>
     </row>
@@ -2155,21 +2155,21 @@
         <v>71</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>46128</v>
+        <v>46126</v>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -2178,11 +2178,11 @@
         <v>72</v>
       </c>
       <c r="B74" s="8" t="n">
-        <v>46129</v>
+        <v>46127</v>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -2201,21 +2201,21 @@
         <v>73</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>46130</v>
+        <v>46128</v>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Bisu</t>
         </is>
       </c>
     </row>
@@ -2224,21 +2224,21 @@
         <v>74</v>
       </c>
       <c r="B76" s="8" t="n">
-        <v>46131</v>
+        <v>46129</v>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>1:4</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Effort</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -2247,21 +2247,21 @@
         <v>75</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>46132</v>
+        <v>46130</v>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -2270,21 +2270,21 @@
         <v>76</v>
       </c>
       <c r="B78" s="8" t="n">
-        <v>46132</v>
+        <v>46131</v>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>Effort</t>
         </is>
       </c>
     </row>
@@ -2293,21 +2293,21 @@
         <v>77</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>46133</v>
+        <v>46132</v>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -2316,21 +2316,21 @@
         <v>78</v>
       </c>
       <c r="B80" s="8" t="n">
-        <v>46134</v>
+        <v>46132</v>
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -2339,21 +2339,21 @@
         <v>79</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>46135</v>
+        <v>46133</v>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -2362,21 +2362,21 @@
         <v>80</v>
       </c>
       <c r="B82" s="8" t="n">
-        <v>46136</v>
+        <v>46134</v>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Best</t>
         </is>
       </c>
     </row>
@@ -2385,21 +2385,21 @@
         <v>81</v>
       </c>
       <c r="B83" s="4" t="n">
-        <v>46137</v>
+        <v>46135</v>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>Tulbo</t>
+          <t>Best</t>
         </is>
       </c>
     </row>
@@ -2408,21 +2408,21 @@
         <v>82</v>
       </c>
       <c r="B84" s="8" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Tulbo</t>
+          <t>Action</t>
         </is>
       </c>
     </row>
@@ -2431,11 +2431,11 @@
         <v>83</v>
       </c>
       <c r="B85" s="4" t="n">
-        <v>46138</v>
+        <v>46137</v>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Tulbo</t>
         </is>
       </c>
     </row>
@@ -2454,11 +2454,11 @@
         <v>84</v>
       </c>
       <c r="B86" s="8" t="n">
-        <v>46138</v>
+        <v>46137</v>
       </c>
       <c r="C86" s="9" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Tulbo</t>
         </is>
       </c>
     </row>
@@ -2477,11 +2477,11 @@
         <v>85</v>
       </c>
       <c r="B87" s="4" t="n">
-        <v>46139</v>
+        <v>46138</v>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>Effort</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -2500,21 +2500,21 @@
         <v>86</v>
       </c>
       <c r="B88" s="8" t="n">
-        <v>46140</v>
+        <v>46138</v>
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -2523,21 +2523,21 @@
         <v>87</v>
       </c>
       <c r="B89" s="4" t="n">
-        <v>46141</v>
+        <v>46139</v>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Effort</t>
         </is>
       </c>
     </row>
@@ -2546,11 +2546,11 @@
         <v>88</v>
       </c>
       <c r="B90" s="8" t="n">
-        <v>46142</v>
+        <v>46140</v>
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
@@ -2569,7 +2569,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="4" t="n">
-        <v>46142</v>
+        <v>46141</v>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
@@ -2578,12 +2578,12 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -2592,21 +2592,21 @@
         <v>90</v>
       </c>
       <c r="B92" s="8" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
+          <t>sSak</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="inlineStr">
+        <is>
           <t>JD</t>
-        </is>
-      </c>
-      <c r="D92" s="10" t="inlineStr">
-        <is>
-          <t>1:4</t>
-        </is>
-      </c>
-      <c r="E92" s="9" t="inlineStr">
-        <is>
-          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -2615,21 +2615,21 @@
         <v>91</v>
       </c>
       <c r="B93" s="4" t="n">
-        <v>46144</v>
+        <v>46142</v>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -2638,21 +2638,21 @@
         <v>92</v>
       </c>
       <c r="B94" s="8" t="n">
-        <v>46145</v>
+        <v>46143</v>
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>1:4</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -2661,21 +2661,21 @@
         <v>93</v>
       </c>
       <c r="B95" s="4" t="n">
-        <v>46146</v>
+        <v>46144</v>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>Soulkey</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
         <v>94</v>
       </c>
       <c r="B96" s="8" t="n">
-        <v>46147</v>
+        <v>46145</v>
       </c>
       <c r="C96" s="9" t="inlineStr">
         <is>
@@ -2693,12 +2693,12 @@
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Rush</t>
         </is>
       </c>
     </row>
@@ -2707,21 +2707,21 @@
         <v>95</v>
       </c>
       <c r="B97" s="4" t="n">
-        <v>46148</v>
+        <v>46146</v>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Soulkey</t>
         </is>
       </c>
     </row>
@@ -2730,11 +2730,11 @@
         <v>96</v>
       </c>
       <c r="B98" s="8" t="n">
-        <v>46152</v>
+        <v>46147</v>
       </c>
       <c r="C98" s="9" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -2753,11 +2753,11 @@
         <v>97</v>
       </c>
       <c r="B99" s="4" t="n">
-        <v>46153</v>
+        <v>46148</v>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>Soulkey</t>
+          <t>Light</t>
         </is>
       </c>
     </row>
@@ -2776,21 +2776,21 @@
         <v>98</v>
       </c>
       <c r="B100" s="8" t="n">
-        <v>46154</v>
+        <v>46152</v>
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Sorry</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -2799,21 +2799,21 @@
         <v>99</v>
       </c>
       <c r="B101" s="4" t="n">
-        <v>46154</v>
+        <v>46153</v>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Soulkey</t>
         </is>
       </c>
     </row>
@@ -2822,21 +2822,21 @@
         <v>100</v>
       </c>
       <c r="B102" s="8" t="n">
-        <v>46155</v>
+        <v>46154</v>
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -2845,21 +2845,21 @@
         <v>101</v>
       </c>
       <c r="B103" s="4" t="n">
-        <v>46156</v>
+        <v>46154</v>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
+          <t>Best</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
           <t>JD</t>
-        </is>
-      </c>
-      <c r="D103" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E103" s="5" t="inlineStr">
-        <is>
-          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -2868,11 +2868,11 @@
         <v>102</v>
       </c>
       <c r="B104" s="8" t="n">
-        <v>46157</v>
+        <v>46155</v>
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -2891,21 +2891,21 @@
         <v>103</v>
       </c>
       <c r="B105" s="4" t="n">
-        <v>46158</v>
+        <v>46156</v>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>1:4</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -2914,11 +2914,11 @@
         <v>104</v>
       </c>
       <c r="B106" s="8" t="n">
-        <v>46159</v>
+        <v>46157</v>
       </c>
       <c r="C106" s="9" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Best</t>
         </is>
       </c>
     </row>
@@ -2937,21 +2937,21 @@
         <v>105</v>
       </c>
       <c r="B107" s="4" t="n">
-        <v>46160</v>
+        <v>46158</v>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>1:4</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>Effort</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -2960,21 +2960,21 @@
         <v>106</v>
       </c>
       <c r="B108" s="8" t="n">
-        <v>46161</v>
+        <v>46159</v>
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -2983,7 +2983,7 @@
         <v>107</v>
       </c>
       <c r="B109" s="4" t="n">
-        <v>46161</v>
+        <v>46160</v>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
@@ -2992,12 +2992,12 @@
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Effort</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3006,7 @@
         <v>108</v>
       </c>
       <c r="B110" s="8" t="n">
-        <v>46162</v>
+        <v>46161</v>
       </c>
       <c r="C110" s="9" t="inlineStr">
         <is>
@@ -3015,12 +3015,12 @@
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
         <v>109</v>
       </c>
       <c r="B111" s="4" t="n">
-        <v>46163</v>
+        <v>46161</v>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
@@ -3038,12 +3038,12 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -3052,21 +3052,21 @@
         <v>110</v>
       </c>
       <c r="B112" s="8" t="n">
-        <v>46164</v>
+        <v>46162</v>
       </c>
       <c r="C112" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -3075,21 +3075,21 @@
         <v>111</v>
       </c>
       <c r="B113" s="4" t="n">
-        <v>46165</v>
+        <v>46163</v>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Mong</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -3098,21 +3098,21 @@
         <v>112</v>
       </c>
       <c r="B114" s="8" t="n">
-        <v>46165</v>
+        <v>46164</v>
       </c>
       <c r="C114" s="9" t="inlineStr">
         <is>
-          <t>Mong</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -3121,21 +3121,21 @@
         <v>113</v>
       </c>
       <c r="B115" s="4" t="n">
-        <v>46167</v>
+        <v>46165</v>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Mong</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -3144,21 +3144,21 @@
         <v>114</v>
       </c>
       <c r="B116" s="8" t="n">
-        <v>46176</v>
+        <v>46165</v>
       </c>
       <c r="C116" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Mong</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E116" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -3167,16 +3167,16 @@
         <v>115</v>
       </c>
       <c r="B117" s="4" t="n">
-        <v>46178</v>
+        <v>46167</v>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
@@ -3190,21 +3190,21 @@
         <v>116</v>
       </c>
       <c r="B118" s="8" t="n">
-        <v>46179</v>
+        <v>46176</v>
       </c>
       <c r="C118" s="9" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t>2:4</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E118" s="9" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -3213,11 +3213,11 @@
         <v>117</v>
       </c>
       <c r="B119" s="4" t="n">
-        <v>46180</v>
+        <v>46178</v>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -3236,21 +3236,21 @@
         <v>118</v>
       </c>
       <c r="B120" s="8" t="n">
-        <v>46181</v>
+        <v>46179</v>
       </c>
       <c r="C120" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="E120" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -3259,11 +3259,11 @@
         <v>119</v>
       </c>
       <c r="B121" s="4" t="n">
-        <v>46182</v>
+        <v>46180</v>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Snow</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Stork</t>
         </is>
       </c>
     </row>
@@ -3282,11 +3282,11 @@
         <v>120</v>
       </c>
       <c r="B122" s="8" t="n">
-        <v>46183</v>
+        <v>46181</v>
       </c>
       <c r="C122" s="9" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="E122" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -3305,21 +3305,21 @@
         <v>121</v>
       </c>
       <c r="B123" s="4" t="n">
-        <v>46184</v>
+        <v>46182</v>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>Snow</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Rush</t>
         </is>
       </c>
     </row>
@@ -3328,11 +3328,11 @@
         <v>122</v>
       </c>
       <c r="B124" s="8" t="n">
-        <v>46185</v>
+        <v>46183</v>
       </c>
       <c r="C124" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="E124" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -3351,21 +3351,21 @@
         <v>123</v>
       </c>
       <c r="B125" s="4" t="n">
-        <v>46186</v>
+        <v>46184</v>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Stork</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -3374,21 +3374,21 @@
         <v>124</v>
       </c>
       <c r="B126" s="8" t="n">
-        <v>46187</v>
+        <v>46185</v>
       </c>
       <c r="C126" s="9" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E126" s="9" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -3397,21 +3397,21 @@
         <v>125</v>
       </c>
       <c r="B127" s="4" t="n">
-        <v>46187</v>
+        <v>46186</v>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Soma</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -3420,21 +3420,21 @@
         <v>126</v>
       </c>
       <c r="B128" s="8" t="n">
-        <v>46188</v>
+        <v>46187</v>
       </c>
       <c r="C128" s="9" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E128" s="9" t="inlineStr">
         <is>
-          <t>Snow</t>
+          <t>Stork</t>
         </is>
       </c>
     </row>
@@ -3443,21 +3443,21 @@
         <v>127</v>
       </c>
       <c r="B129" s="4" t="n">
-        <v>46189</v>
+        <v>46187</v>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Stork</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
         <v>128</v>
       </c>
       <c r="B130" s="8" t="n">
-        <v>46190</v>
+        <v>46188</v>
       </c>
       <c r="C130" s="9" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="E130" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Snow</t>
         </is>
       </c>
     </row>
@@ -3489,21 +3489,21 @@
         <v>129</v>
       </c>
       <c r="B131" s="4" t="n">
-        <v>46191</v>
+        <v>46189</v>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Leta</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>1:4</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -3512,21 +3512,21 @@
         <v>130</v>
       </c>
       <c r="B132" s="8" t="n">
-        <v>46192</v>
+        <v>46190</v>
       </c>
       <c r="C132" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E132" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Best</t>
         </is>
       </c>
     </row>
@@ -3535,21 +3535,21 @@
         <v>131</v>
       </c>
       <c r="B133" s="4" t="n">
-        <v>46193</v>
+        <v>46191</v>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Leta</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>1:4</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Stork</t>
         </is>
       </c>
     </row>
@@ -3558,21 +3558,21 @@
         <v>132</v>
       </c>
       <c r="B134" s="8" t="n">
-        <v>46194</v>
+        <v>46192</v>
       </c>
       <c r="C134" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E134" s="9" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -3581,21 +3581,21 @@
         <v>133</v>
       </c>
       <c r="B135" s="4" t="n">
-        <v>46195</v>
+        <v>46193</v>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Soma</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>2:4</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -3604,21 +3604,21 @@
         <v>134</v>
       </c>
       <c r="B136" s="8" t="n">
-        <v>46196</v>
+        <v>46194</v>
       </c>
       <c r="C136" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t>1:4</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E136" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -3627,21 +3627,21 @@
         <v>135</v>
       </c>
       <c r="B137" s="4" t="n">
-        <v>46196</v>
+        <v>46195</v>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3650,7 @@
         <v>136</v>
       </c>
       <c r="B138" s="8" t="n">
-        <v>46197</v>
+        <v>46196</v>
       </c>
       <c r="C138" s="9" t="inlineStr">
         <is>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t>2:4</t>
+          <t>1:4</t>
         </is>
       </c>
       <c r="E138" s="9" t="inlineStr">
@@ -3673,21 +3673,21 @@
         <v>137</v>
       </c>
       <c r="B139" s="4" t="n">
-        <v>46202</v>
+        <v>46196</v>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -3696,7 +3696,7 @@
         <v>138</v>
       </c>
       <c r="B140" s="8" t="n">
-        <v>46203</v>
+        <v>46197</v>
       </c>
       <c r="C140" s="9" t="inlineStr">
         <is>
@@ -3705,12 +3705,12 @@
       </c>
       <c r="D140" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="E140" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -3719,21 +3719,21 @@
         <v>139</v>
       </c>
       <c r="B141" s="4" t="n">
-        <v>46204</v>
+        <v>46202</v>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -3742,21 +3742,21 @@
         <v>140</v>
       </c>
       <c r="B142" s="8" t="n">
-        <v>46205</v>
+        <v>46203</v>
       </c>
       <c r="C142" s="9" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D142" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E142" s="9" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Rush</t>
         </is>
       </c>
     </row>
@@ -3765,21 +3765,21 @@
         <v>141</v>
       </c>
       <c r="B143" s="4" t="n">
-        <v>46207</v>
+        <v>46204</v>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t>Mong</t>
+          <t>Rush</t>
         </is>
       </c>
     </row>
@@ -3788,21 +3788,21 @@
         <v>142</v>
       </c>
       <c r="B144" s="8" t="n">
-        <v>46207</v>
+        <v>46205</v>
       </c>
       <c r="C144" s="9" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Soma</t>
         </is>
       </c>
       <c r="D144" s="10" t="inlineStr">
         <is>
-          <t>3:2</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E144" s="9" t="inlineStr">
         <is>
-          <t>Noob</t>
+          <t>Light</t>
         </is>
       </c>
     </row>
@@ -3811,21 +3811,21 @@
         <v>143</v>
       </c>
       <c r="B145" s="4" t="n">
-        <v>46208</v>
+        <v>46207</v>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Stork</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Mong</t>
         </is>
       </c>
     </row>
@@ -3834,21 +3834,21 @@
         <v>144</v>
       </c>
       <c r="B146" s="8" t="n">
-        <v>46209</v>
+        <v>46207</v>
       </c>
       <c r="C146" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>sSak</t>
         </is>
       </c>
       <c r="D146" s="10" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>3:2</t>
         </is>
       </c>
       <c r="E146" s="9" t="inlineStr">
         <is>
-          <t>sSak</t>
+          <t>Noob</t>
         </is>
       </c>
     </row>
@@ -3857,21 +3857,21 @@
         <v>145</v>
       </c>
       <c r="B147" s="4" t="n">
-        <v>46210</v>
+        <v>46208</v>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -3880,21 +3880,21 @@
         <v>146</v>
       </c>
       <c r="B148" s="8" t="n">
-        <v>46211</v>
+        <v>46209</v>
       </c>
       <c r="C148" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D148" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E148" s="9" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>sSak</t>
         </is>
       </c>
     </row>
@@ -3903,21 +3903,21 @@
         <v>147</v>
       </c>
       <c r="B149" s="4" t="n">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>侠义</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t>爆炸头</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -3926,21 +3926,21 @@
         <v>148</v>
       </c>
       <c r="B150" s="8" t="n">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="C150" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D150" s="10" t="inlineStr">
         <is>
-          <t>2:4</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E150" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Light</t>
         </is>
       </c>
     </row>
@@ -3949,21 +3949,21 @@
         <v>149</v>
       </c>
       <c r="B151" s="4" t="n">
-        <v>46214</v>
+        <v>46211</v>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>侠义</t>
         </is>
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>1:3</t>
         </is>
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t>Tyson</t>
+          <t>爆炸头</t>
         </is>
       </c>
     </row>
@@ -3972,21 +3972,21 @@
         <v>150</v>
       </c>
       <c r="B152" s="8" t="n">
-        <v>46214</v>
+        <v>46212</v>
       </c>
       <c r="C152" s="9" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D152" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="E152" s="9" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -3995,21 +3995,21 @@
         <v>151</v>
       </c>
       <c r="B153" s="4" t="n">
-        <v>46215</v>
+        <v>46214</v>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Sharp</t>
         </is>
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Tyson</t>
         </is>
       </c>
     </row>
@@ -4018,21 +4018,21 @@
         <v>152</v>
       </c>
       <c r="B154" s="8" t="n">
-        <v>46216</v>
+        <v>46214</v>
       </c>
       <c r="C154" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Sharp</t>
         </is>
       </c>
       <c r="D154" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E154" s="9" t="inlineStr">
         <is>
-          <t>解冻</t>
+          <t>Stork</t>
         </is>
       </c>
     </row>
@@ -4041,11 +4041,11 @@
         <v>153</v>
       </c>
       <c r="B155" s="4" t="n">
-        <v>46217</v>
+        <v>46215</v>
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D155" s="6" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4064,7 @@
         <v>154</v>
       </c>
       <c r="B156" s="8" t="n">
-        <v>46218</v>
+        <v>46216</v>
       </c>
       <c r="C156" s="9" t="inlineStr">
         <is>
@@ -4073,12 +4073,12 @@
       </c>
       <c r="D156" s="10" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E156" s="9" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>解冻</t>
         </is>
       </c>
     </row>
@@ -4087,11 +4087,11 @@
         <v>155</v>
       </c>
       <c r="B157" s="4" t="n">
-        <v>46219</v>
+        <v>46217</v>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D157" s="6" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Speed</t>
         </is>
       </c>
     </row>
@@ -4110,21 +4110,21 @@
         <v>156</v>
       </c>
       <c r="B158" s="8" t="n">
-        <v>46222</v>
+        <v>46218</v>
       </c>
       <c r="C158" s="9" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D158" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E158" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Sorry</t>
         </is>
       </c>
     </row>
@@ -4133,21 +4133,21 @@
         <v>157</v>
       </c>
       <c r="B159" s="4" t="n">
-        <v>46223</v>
+        <v>46219</v>
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -4156,11 +4156,11 @@
         <v>158</v>
       </c>
       <c r="B160" s="8" t="n">
-        <v>46224</v>
+        <v>46222</v>
       </c>
       <c r="C160" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Sharp</t>
         </is>
       </c>
       <c r="D160" s="10" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="E160" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -4179,16 +4179,16 @@
         <v>159</v>
       </c>
       <c r="B161" s="4" t="n">
-        <v>46225</v>
+        <v>46223</v>
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E161" s="5" t="inlineStr">
@@ -4202,21 +4202,21 @@
         <v>160</v>
       </c>
       <c r="B162" s="8" t="n">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="C162" s="9" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D162" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E162" s="9" t="inlineStr">
         <is>
-          <t>Stork</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -4225,21 +4225,21 @@
         <v>161</v>
       </c>
       <c r="B163" s="4" t="n">
-        <v>46227</v>
+        <v>46225</v>
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -4248,21 +4248,21 @@
         <v>162</v>
       </c>
       <c r="B164" s="8" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="C164" s="9" t="inlineStr">
         <is>
-          <t>侠义</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="D164" s="10" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E164" s="9" t="inlineStr">
         <is>
-          <t>爆炸头</t>
+          <t>Stork</t>
         </is>
       </c>
     </row>
@@ -4271,21 +4271,21 @@
         <v>163</v>
       </c>
       <c r="B165" s="4" t="n">
-        <v>46228</v>
+        <v>46227</v>
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Soma</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Light</t>
         </is>
       </c>
     </row>
@@ -4294,21 +4294,21 @@
         <v>164</v>
       </c>
       <c r="B166" s="8" t="n">
-        <v>46229</v>
+        <v>46227</v>
       </c>
       <c r="C166" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>侠义</t>
         </is>
       </c>
       <c r="D166" s="10" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>3:0</t>
         </is>
       </c>
       <c r="E166" s="9" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>爆炸头</t>
         </is>
       </c>
     </row>
@@ -4317,21 +4317,21 @@
         <v>165</v>
       </c>
       <c r="B167" s="4" t="n">
-        <v>46230</v>
+        <v>46228</v>
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>1:4</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Speed</t>
         </is>
       </c>
     </row>
@@ -4340,21 +4340,21 @@
         <v>166</v>
       </c>
       <c r="B168" s="8" t="n">
-        <v>46230</v>
+        <v>46229</v>
       </c>
       <c r="C168" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D168" s="10" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E168" s="9" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Speed</t>
         </is>
       </c>
     </row>
@@ -4363,21 +4363,21 @@
         <v>167</v>
       </c>
       <c r="B169" s="4" t="n">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>1:4</t>
         </is>
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -4386,7 +4386,7 @@
         <v>168</v>
       </c>
       <c r="B170" s="8" t="n">
-        <v>46232</v>
+        <v>46230</v>
       </c>
       <c r="C170" s="9" t="inlineStr">
         <is>
@@ -4395,12 +4395,12 @@
       </c>
       <c r="D170" s="10" t="inlineStr">
         <is>
-          <t>0:4</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E170" s="9" t="inlineStr">
         <is>
-          <t>Soulkey</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -4409,21 +4409,21 @@
         <v>169</v>
       </c>
       <c r="B171" s="4" t="n">
-        <v>46232</v>
+        <v>46231</v>
       </c>
       <c r="C171" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>Soulkey</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
         <v>170</v>
       </c>
       <c r="B172" s="8" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="C172" s="9" t="inlineStr">
         <is>
@@ -4441,12 +4441,12 @@
       </c>
       <c r="D172" s="10" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>0:4</t>
         </is>
       </c>
       <c r="E172" s="9" t="inlineStr">
         <is>
-          <t>HBQ</t>
+          <t>Soulkey</t>
         </is>
       </c>
     </row>
@@ -4455,7 +4455,7 @@
         <v>171</v>
       </c>
       <c r="B173" s="4" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="C173" s="5" t="inlineStr">
         <is>
@@ -4464,12 +4464,12 @@
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Soulkey</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
         <v>172</v>
       </c>
       <c r="B174" s="8" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="C174" s="9" t="inlineStr">
         <is>
@@ -4487,12 +4487,12 @@
       </c>
       <c r="D174" s="10" t="inlineStr">
         <is>
-          <t>1:4</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="E174" s="9" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>HBQ</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
         <v>173</v>
       </c>
       <c r="B175" s="4" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="C175" s="5" t="inlineStr">
         <is>
@@ -4510,12 +4510,12 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -4524,21 +4524,21 @@
         <v>174</v>
       </c>
       <c r="B176" s="8" t="n">
-        <v>46244</v>
+        <v>46241</v>
       </c>
       <c r="C176" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D176" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>1:4</t>
         </is>
       </c>
       <c r="E176" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -4547,16 +4547,16 @@
         <v>175</v>
       </c>
       <c r="B177" s="4" t="n">
-        <v>46249</v>
+        <v>46241</v>
       </c>
       <c r="C177" s="5" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="E177" s="5" t="inlineStr">
@@ -4570,7 +4570,7 @@
         <v>176</v>
       </c>
       <c r="B178" s="8" t="n">
-        <v>46250</v>
+        <v>46244</v>
       </c>
       <c r="C178" s="9" t="inlineStr">
         <is>
@@ -4579,12 +4579,12 @@
       </c>
       <c r="D178" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E178" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -4593,21 +4593,21 @@
         <v>177</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>46251</v>
+        <v>46249</v>
       </c>
       <c r="C179" s="5" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Soma</t>
         </is>
       </c>
     </row>
@@ -4616,21 +4616,21 @@
         <v>178</v>
       </c>
       <c r="B180" s="8" t="n">
-        <v>46252</v>
+        <v>46250</v>
       </c>
       <c r="C180" s="9" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D180" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E180" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Rush</t>
         </is>
       </c>
     </row>
@@ -4639,11 +4639,11 @@
         <v>179</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="C181" s="5" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="D181" s="6" t="inlineStr">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
-          <t>Effort</t>
+          <t>Speed</t>
         </is>
       </c>
     </row>
@@ -4662,21 +4662,21 @@
         <v>180</v>
       </c>
       <c r="B182" s="8" t="n">
-        <v>46256</v>
+        <v>46252</v>
       </c>
       <c r="C182" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Soma</t>
         </is>
       </c>
       <c r="D182" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E182" s="9" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Best</t>
         </is>
       </c>
     </row>
@@ -4685,21 +4685,21 @@
         <v>181</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>46257</v>
+        <v>46253</v>
       </c>
       <c r="C183" s="5" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Effort</t>
         </is>
       </c>
     </row>
@@ -4708,21 +4708,21 @@
         <v>182</v>
       </c>
       <c r="B184" s="8" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="C184" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="D184" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E184" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Speed</t>
         </is>
       </c>
     </row>
@@ -4731,16 +4731,16 @@
         <v>183</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="C185" s="5" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Sharp</t>
         </is>
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E185" s="5" t="inlineStr">
@@ -4754,21 +4754,21 @@
         <v>184</v>
       </c>
       <c r="B186" s="8" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="C186" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D186" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E186" s="9" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -4777,21 +4777,21 @@
         <v>185</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="C187" s="5" t="inlineStr">
         <is>
-          <t>Mihu</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>0:4</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E187" s="5" t="inlineStr">
         <is>
-          <t>Effort</t>
+          <t>Bisu</t>
         </is>
       </c>
     </row>
@@ -4800,21 +4800,21 @@
         <v>186</v>
       </c>
       <c r="B188" s="8" t="n">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="C188" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D188" s="10" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E188" s="9" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -4823,21 +4823,21 @@
         <v>187</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="C189" s="5" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>Mihu</t>
         </is>
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>2:4</t>
+          <t>0:4</t>
         </is>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Effort</t>
         </is>
       </c>
     </row>
@@ -4846,21 +4846,21 @@
         <v>188</v>
       </c>
       <c r="B190" s="8" t="n">
-        <v>46264</v>
+        <v>46262</v>
       </c>
       <c r="C190" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="D190" s="10" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E190" s="9" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Best</t>
         </is>
       </c>
     </row>
@@ -4869,11 +4869,11 @@
         <v>189</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>46265</v>
+        <v>46263</v>
       </c>
       <c r="C191" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="D191" s="6" t="inlineStr">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="E191" s="5" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Speed</t>
         </is>
       </c>
     </row>
@@ -4892,11 +4892,11 @@
         <v>190</v>
       </c>
       <c r="B192" s="8" t="n">
-        <v>46266</v>
+        <v>46264</v>
       </c>
       <c r="C192" s="9" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D192" s="10" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="E192" s="9" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>JD</t>
         </is>
       </c>
     </row>
@@ -4915,7 +4915,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="C193" s="5" t="inlineStr">
         <is>
@@ -4924,12 +4924,12 @@
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="E193" s="5" t="inlineStr">
         <is>
-          <t>Soulkey</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -4938,21 +4938,21 @@
         <v>192</v>
       </c>
       <c r="B194" s="8" t="n">
-        <v>46268</v>
+        <v>46266</v>
       </c>
       <c r="C194" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="D194" s="10" t="inlineStr">
         <is>
-          <t>4:3</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E194" s="9" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Rush</t>
         </is>
       </c>
     </row>
@@ -4961,21 +4961,21 @@
         <v>193</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>46269</v>
+        <v>46267</v>
       </c>
       <c r="C195" s="5" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>2:4</t>
+          <t>3:4</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Soulkey</t>
         </is>
       </c>
     </row>
@@ -4984,11 +4984,11 @@
         <v>194</v>
       </c>
       <c r="B196" s="8" t="n">
-        <v>46271</v>
+        <v>46268</v>
       </c>
       <c r="C196" s="9" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D196" s="10" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="E196" s="9" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -5007,21 +5007,21 @@
         <v>195</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>46272</v>
+        <v>46269</v>
       </c>
       <c r="C197" s="5" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Queen</t>
         </is>
       </c>
     </row>
@@ -5030,11 +5030,11 @@
         <v>196</v>
       </c>
       <c r="B198" s="8" t="n">
-        <v>46273</v>
+        <v>46271</v>
       </c>
       <c r="C198" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="D198" s="10" t="inlineStr">
@@ -5053,7 +5053,7 @@
         <v>197</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>46274</v>
+        <v>46272</v>
       </c>
       <c r="C199" s="5" t="inlineStr">
         <is>
@@ -5062,12 +5062,12 @@
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
         <is>
-          <t>Mini</t>
+          <t>Bisu</t>
         </is>
       </c>
     </row>
@@ -5076,11 +5076,11 @@
         <v>198</v>
       </c>
       <c r="B200" s="8" t="n">
-        <v>46275</v>
+        <v>46273</v>
       </c>
       <c r="C200" s="9" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Bisu</t>
         </is>
       </c>
       <c r="D200" s="10" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="E200" s="9" t="inlineStr">
         <is>
-          <t>Soulkey</t>
+          <t>Hero</t>
         </is>
       </c>
     </row>
@@ -5099,11 +5099,11 @@
         <v>199</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>46277</v>
+        <v>46274</v>
       </c>
       <c r="C201" s="5" t="inlineStr">
         <is>
-          <t>Sorry</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="D201" s="6" t="inlineStr">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="E201" s="5" t="inlineStr">
         <is>
-          <t>Soulkey</t>
+          <t>Mini</t>
         </is>
       </c>
     </row>
@@ -5122,11 +5122,11 @@
         <v>200</v>
       </c>
       <c r="B202" s="8" t="n">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="C202" s="9" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Sharp</t>
         </is>
       </c>
       <c r="D202" s="10" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="E202" s="9" t="inlineStr">
         <is>
-          <t>Sharp</t>
+          <t>Soulkey</t>
         </is>
       </c>
     </row>
@@ -5145,21 +5145,21 @@
         <v>201</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="C203" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Sorry</t>
         </is>
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Soulkey</t>
         </is>
       </c>
     </row>
@@ -5168,21 +5168,21 @@
         <v>202</v>
       </c>
       <c r="B204" s="8" t="n">
-        <v>46280</v>
+        <v>46278</v>
       </c>
       <c r="C204" s="9" t="inlineStr">
         <is>
-          <t>Bisu</t>
+          <t>Soma</t>
         </is>
       </c>
       <c r="D204" s="10" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>4:3</t>
         </is>
       </c>
       <c r="E204" s="9" t="inlineStr">
         <is>
-          <t>Soma</t>
+          <t>Sharp</t>
         </is>
       </c>
     </row>
@@ -5191,16 +5191,16 @@
         <v>203</v>
       </c>
       <c r="B205" s="4" t="n">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="C205" s="5" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>4:2</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="E205" s="5" t="inlineStr">
@@ -5214,26 +5214,95 @@
         <v>204</v>
       </c>
       <c r="B206" s="8" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C206" s="9" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D206" s="10" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E206" s="9" t="inlineStr">
+        <is>
+          <t>Soma</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="n">
+        <v>205</v>
+      </c>
+      <c r="B207" s="4" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>Rush</t>
+        </is>
+      </c>
+      <c r="D207" s="6" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="7" t="n">
+        <v>206</v>
+      </c>
+      <c r="B208" s="8" t="n">
         <v>46283</v>
       </c>
-      <c r="C206" s="9" t="inlineStr">
+      <c r="C208" s="9" t="inlineStr">
         <is>
           <t>Stork</t>
         </is>
       </c>
-      <c r="D206" s="10" t="inlineStr">
+      <c r="D208" s="10" t="inlineStr">
         <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="E206" s="9" t="inlineStr">
+      <c r="E208" s="9" t="inlineStr">
         <is>
           <t>迷糊</t>
         </is>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" s="3" t="n">
+        <v>207</v>
+      </c>
+      <c r="B209" s="4" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C209" s="5" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="D209" s="6" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>JD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E206"/>
+  <autoFilter ref="A2:E209"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5281,7 +5350,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-01-01 至 2026-09-18，共 204 场「巅峰赛场」对局。</t>
+          <t>2026-01-01 至 2026-09-18，共 207 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-09-22（共 210 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$209</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$212</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E209"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5301,8 +5301,77 @@
         </is>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" s="7" t="n">
+        <v>208</v>
+      </c>
+      <c r="B210" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="C210" s="9" t="inlineStr">
+        <is>
+          <t>Sharp</t>
+        </is>
+      </c>
+      <c r="D210" s="10" t="inlineStr">
+        <is>
+          <t>4:3</t>
+        </is>
+      </c>
+      <c r="E210" s="9" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="n">
+        <v>209</v>
+      </c>
+      <c r="B211" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C211" s="5" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="D211" s="6" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
+      <c r="E211" s="5" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="B212" s="8" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C212" s="9" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="D212" s="10" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
+      <c r="E212" s="9" t="inlineStr">
+        <is>
+          <t>Hero</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E209"/>
+  <autoFilter ref="A2:E212"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5350,7 +5419,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-01-01 至 2026-09-18，共 207 场「巅峰赛场」对局。</t>
+          <t>2026-01-01 至 2026-09-18，共 210 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-09-25（共 213 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$215</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E212"/>
+  <dimension ref="A1:E215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5370,8 +5370,77 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" s="3" t="n">
+        <v>211</v>
+      </c>
+      <c r="B213" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C213" s="5" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+      <c r="D213" s="6" t="inlineStr">
+        <is>
+          <t>4:3</t>
+        </is>
+      </c>
+      <c r="E213" s="5" t="inlineStr">
+        <is>
+          <t>Sorry</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="7" t="n">
+        <v>212</v>
+      </c>
+      <c r="B214" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C214" s="9" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D214" s="10" t="inlineStr">
+        <is>
+          <t>2:4</t>
+        </is>
+      </c>
+      <c r="E214" s="9" t="inlineStr">
+        <is>
+          <t>Soulkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="3" t="n">
+        <v>213</v>
+      </c>
+      <c r="B215" s="4" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C215" s="5" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D215" s="6" t="inlineStr">
+        <is>
+          <t>0:4</t>
+        </is>
+      </c>
+      <c r="E215" s="5" t="inlineStr">
+        <is>
+          <t>JD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E212"/>
+  <autoFilter ref="A2:E215"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5419,7 +5488,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-01-01 至 2026-09-18，共 210 场「巅峰赛场」对局。</t>
+          <t>2026-01-01 至 2026-09-18，共 213 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-06-29（共 139 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$215</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E215"/>
+  <dimension ref="A1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3737,1710 +3737,8 @@
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="7" t="n">
-        <v>140</v>
-      </c>
-      <c r="B142" s="8" t="n">
-        <v>46203</v>
-      </c>
-      <c r="C142" s="9" t="inlineStr">
-        <is>
-          <t>Mini</t>
-        </is>
-      </c>
-      <c r="D142" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E142" s="9" t="inlineStr">
-        <is>
-          <t>Rush</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="3" t="n">
-        <v>141</v>
-      </c>
-      <c r="B143" s="4" t="n">
-        <v>46204</v>
-      </c>
-      <c r="C143" s="5" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D143" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E143" s="5" t="inlineStr">
-        <is>
-          <t>Rush</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="7" t="n">
-        <v>142</v>
-      </c>
-      <c r="B144" s="8" t="n">
-        <v>46205</v>
-      </c>
-      <c r="C144" s="9" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-      <c r="D144" s="10" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E144" s="9" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="3" t="n">
-        <v>143</v>
-      </c>
-      <c r="B145" s="4" t="n">
-        <v>46207</v>
-      </c>
-      <c r="C145" s="5" t="inlineStr">
-        <is>
-          <t>Stork</t>
-        </is>
-      </c>
-      <c r="D145" s="6" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E145" s="5" t="inlineStr">
-        <is>
-          <t>Mong</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="7" t="n">
-        <v>144</v>
-      </c>
-      <c r="B146" s="8" t="n">
-        <v>46207</v>
-      </c>
-      <c r="C146" s="9" t="inlineStr">
-        <is>
-          <t>sSak</t>
-        </is>
-      </c>
-      <c r="D146" s="10" t="inlineStr">
-        <is>
-          <t>3:2</t>
-        </is>
-      </c>
-      <c r="E146" s="9" t="inlineStr">
-        <is>
-          <t>Noob</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="3" t="n">
-        <v>145</v>
-      </c>
-      <c r="B147" s="4" t="n">
-        <v>46208</v>
-      </c>
-      <c r="C147" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D147" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E147" s="5" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="7" t="n">
-        <v>146</v>
-      </c>
-      <c r="B148" s="8" t="n">
-        <v>46209</v>
-      </c>
-      <c r="C148" s="9" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="D148" s="10" t="inlineStr">
-        <is>
-          <t>4:0</t>
-        </is>
-      </c>
-      <c r="E148" s="9" t="inlineStr">
-        <is>
-          <t>sSak</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="3" t="n">
-        <v>147</v>
-      </c>
-      <c r="B149" s="4" t="n">
-        <v>46210</v>
-      </c>
-      <c r="C149" s="5" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="D149" s="6" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E149" s="5" t="inlineStr">
-        <is>
-          <t>Mini</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="7" t="n">
-        <v>148</v>
-      </c>
-      <c r="B150" s="8" t="n">
-        <v>46211</v>
-      </c>
-      <c r="C150" s="9" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D150" s="10" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E150" s="9" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="3" t="n">
-        <v>149</v>
-      </c>
-      <c r="B151" s="4" t="n">
-        <v>46211</v>
-      </c>
-      <c r="C151" s="5" t="inlineStr">
-        <is>
-          <t>侠义</t>
-        </is>
-      </c>
-      <c r="D151" s="6" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
-      <c r="E151" s="5" t="inlineStr">
-        <is>
-          <t>爆炸头</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="7" t="n">
-        <v>150</v>
-      </c>
-      <c r="B152" s="8" t="n">
-        <v>46212</v>
-      </c>
-      <c r="C152" s="9" t="inlineStr">
-        <is>
-          <t>Rush</t>
-        </is>
-      </c>
-      <c r="D152" s="10" t="inlineStr">
-        <is>
-          <t>2:4</t>
-        </is>
-      </c>
-      <c r="E152" s="9" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="3" t="n">
-        <v>151</v>
-      </c>
-      <c r="B153" s="4" t="n">
-        <v>46214</v>
-      </c>
-      <c r="C153" s="5" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-      <c r="D153" s="6" t="inlineStr">
-        <is>
-          <t>3:1</t>
-        </is>
-      </c>
-      <c r="E153" s="5" t="inlineStr">
-        <is>
-          <t>Tyson</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="7" t="n">
-        <v>152</v>
-      </c>
-      <c r="B154" s="8" t="n">
-        <v>46214</v>
-      </c>
-      <c r="C154" s="9" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-      <c r="D154" s="10" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E154" s="9" t="inlineStr">
-        <is>
-          <t>Stork</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="3" t="n">
-        <v>153</v>
-      </c>
-      <c r="B155" s="4" t="n">
-        <v>46215</v>
-      </c>
-      <c r="C155" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D155" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E155" s="5" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="7" t="n">
-        <v>154</v>
-      </c>
-      <c r="B156" s="8" t="n">
-        <v>46216</v>
-      </c>
-      <c r="C156" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D156" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E156" s="9" t="inlineStr">
-        <is>
-          <t>解冻</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="3" t="n">
-        <v>155</v>
-      </c>
-      <c r="B157" s="4" t="n">
-        <v>46217</v>
-      </c>
-      <c r="C157" s="5" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D157" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E157" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="7" t="n">
-        <v>156</v>
-      </c>
-      <c r="B158" s="8" t="n">
-        <v>46218</v>
-      </c>
-      <c r="C158" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D158" s="10" t="inlineStr">
-        <is>
-          <t>4:0</t>
-        </is>
-      </c>
-      <c r="E158" s="9" t="inlineStr">
-        <is>
-          <t>Sorry</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="3" t="n">
-        <v>157</v>
-      </c>
-      <c r="B159" s="4" t="n">
-        <v>46219</v>
-      </c>
-      <c r="C159" s="5" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="D159" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E159" s="5" t="inlineStr">
-        <is>
-          <t>Mini</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="7" t="n">
-        <v>158</v>
-      </c>
-      <c r="B160" s="8" t="n">
-        <v>46222</v>
-      </c>
-      <c r="C160" s="9" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-      <c r="D160" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E160" s="9" t="inlineStr">
-        <is>
-          <t>Mini</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="3" t="n">
-        <v>159</v>
-      </c>
-      <c r="B161" s="4" t="n">
-        <v>46223</v>
-      </c>
-      <c r="C161" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D161" s="6" t="inlineStr">
-        <is>
-          <t>3:4</t>
-        </is>
-      </c>
-      <c r="E161" s="5" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="7" t="n">
-        <v>160</v>
-      </c>
-      <c r="B162" s="8" t="n">
-        <v>46224</v>
-      </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D162" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E162" s="9" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="3" t="n">
-        <v>161</v>
-      </c>
-      <c r="B163" s="4" t="n">
-        <v>46225</v>
-      </c>
-      <c r="C163" s="5" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D163" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E163" s="5" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="7" t="n">
-        <v>162</v>
-      </c>
-      <c r="B164" s="8" t="n">
-        <v>46226</v>
-      </c>
-      <c r="C164" s="9" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="D164" s="10" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E164" s="9" t="inlineStr">
-        <is>
-          <t>Stork</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="3" t="n">
-        <v>163</v>
-      </c>
-      <c r="B165" s="4" t="n">
-        <v>46227</v>
-      </c>
-      <c r="C165" s="5" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-      <c r="D165" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E165" s="5" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="7" t="n">
-        <v>164</v>
-      </c>
-      <c r="B166" s="8" t="n">
-        <v>46227</v>
-      </c>
-      <c r="C166" s="9" t="inlineStr">
-        <is>
-          <t>侠义</t>
-        </is>
-      </c>
-      <c r="D166" s="10" t="inlineStr">
-        <is>
-          <t>3:0</t>
-        </is>
-      </c>
-      <c r="E166" s="9" t="inlineStr">
-        <is>
-          <t>爆炸头</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="3" t="n">
-        <v>165</v>
-      </c>
-      <c r="B167" s="4" t="n">
-        <v>46228</v>
-      </c>
-      <c r="C167" s="5" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D167" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E167" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="7" t="n">
-        <v>166</v>
-      </c>
-      <c r="B168" s="8" t="n">
-        <v>46229</v>
-      </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>Mini</t>
-        </is>
-      </c>
-      <c r="D168" s="10" t="inlineStr">
-        <is>
-          <t>3:4</t>
-        </is>
-      </c>
-      <c r="E168" s="9" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="3" t="n">
-        <v>167</v>
-      </c>
-      <c r="B169" s="4" t="n">
-        <v>46230</v>
-      </c>
-      <c r="C169" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D169" s="6" t="inlineStr">
-        <is>
-          <t>1:4</t>
-        </is>
-      </c>
-      <c r="E169" s="5" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="7" t="n">
-        <v>168</v>
-      </c>
-      <c r="B170" s="8" t="n">
-        <v>46230</v>
-      </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D170" s="10" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="E170" s="9" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="3" t="n">
-        <v>169</v>
-      </c>
-      <c r="B171" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="C171" s="5" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D171" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E171" s="5" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="7" t="n">
-        <v>170</v>
-      </c>
-      <c r="B172" s="8" t="n">
-        <v>46232</v>
-      </c>
-      <c r="C172" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D172" s="10" t="inlineStr">
-        <is>
-          <t>0:4</t>
-        </is>
-      </c>
-      <c r="E172" s="9" t="inlineStr">
-        <is>
-          <t>Soulkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="3" t="n">
-        <v>171</v>
-      </c>
-      <c r="B173" s="4" t="n">
-        <v>46232</v>
-      </c>
-      <c r="C173" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D173" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E173" s="5" t="inlineStr">
-        <is>
-          <t>Soulkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="7" t="n">
-        <v>172</v>
-      </c>
-      <c r="B174" s="8" t="n">
-        <v>46240</v>
-      </c>
-      <c r="C174" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D174" s="10" t="inlineStr">
-        <is>
-          <t>3:1</t>
-        </is>
-      </c>
-      <c r="E174" s="9" t="inlineStr">
-        <is>
-          <t>HBQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="3" t="n">
-        <v>173</v>
-      </c>
-      <c r="B175" s="4" t="n">
-        <v>46240</v>
-      </c>
-      <c r="C175" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D175" s="6" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E175" s="5" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="7" t="n">
-        <v>174</v>
-      </c>
-      <c r="B176" s="8" t="n">
-        <v>46241</v>
-      </c>
-      <c r="C176" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D176" s="10" t="inlineStr">
-        <is>
-          <t>1:4</t>
-        </is>
-      </c>
-      <c r="E176" s="9" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="3" t="n">
-        <v>175</v>
-      </c>
-      <c r="B177" s="4" t="n">
-        <v>46241</v>
-      </c>
-      <c r="C177" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D177" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E177" s="5" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="7" t="n">
-        <v>176</v>
-      </c>
-      <c r="B178" s="8" t="n">
-        <v>46244</v>
-      </c>
-      <c r="C178" s="9" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D178" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E178" s="9" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="3" t="n">
-        <v>177</v>
-      </c>
-      <c r="B179" s="4" t="n">
-        <v>46249</v>
-      </c>
-      <c r="C179" s="5" t="inlineStr">
-        <is>
-          <t>Rush</t>
-        </is>
-      </c>
-      <c r="D179" s="6" t="inlineStr">
-        <is>
-          <t>4:0</t>
-        </is>
-      </c>
-      <c r="E179" s="5" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="7" t="n">
-        <v>178</v>
-      </c>
-      <c r="B180" s="8" t="n">
-        <v>46250</v>
-      </c>
-      <c r="C180" s="9" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D180" s="10" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E180" s="9" t="inlineStr">
-        <is>
-          <t>Rush</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="3" t="n">
-        <v>179</v>
-      </c>
-      <c r="B181" s="4" t="n">
-        <v>46251</v>
-      </c>
-      <c r="C181" s="5" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="D181" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E181" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="7" t="n">
-        <v>180</v>
-      </c>
-      <c r="B182" s="8" t="n">
-        <v>46252</v>
-      </c>
-      <c r="C182" s="9" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-      <c r="D182" s="10" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E182" s="9" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="3" t="n">
-        <v>181</v>
-      </c>
-      <c r="B183" s="4" t="n">
-        <v>46253</v>
-      </c>
-      <c r="C183" s="5" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-      <c r="D183" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E183" s="5" t="inlineStr">
-        <is>
-          <t>Effort</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="7" t="n">
-        <v>182</v>
-      </c>
-      <c r="B184" s="8" t="n">
-        <v>46256</v>
-      </c>
-      <c r="C184" s="9" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-      <c r="D184" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E184" s="9" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="3" t="n">
-        <v>183</v>
-      </c>
-      <c r="B185" s="4" t="n">
-        <v>46257</v>
-      </c>
-      <c r="C185" s="5" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-      <c r="D185" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E185" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="7" t="n">
-        <v>184</v>
-      </c>
-      <c r="B186" s="8" t="n">
-        <v>46258</v>
-      </c>
-      <c r="C186" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D186" s="10" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E186" s="9" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="3" t="n">
-        <v>185</v>
-      </c>
-      <c r="B187" s="4" t="n">
-        <v>46259</v>
-      </c>
-      <c r="C187" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="D187" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E187" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="7" t="n">
-        <v>186</v>
-      </c>
-      <c r="B188" s="8" t="n">
-        <v>46260</v>
-      </c>
-      <c r="C188" s="9" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D188" s="10" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E188" s="9" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="3" t="n">
-        <v>187</v>
-      </c>
-      <c r="B189" s="4" t="n">
-        <v>46261</v>
-      </c>
-      <c r="C189" s="5" t="inlineStr">
-        <is>
-          <t>Mihu</t>
-        </is>
-      </c>
-      <c r="D189" s="6" t="inlineStr">
-        <is>
-          <t>0:4</t>
-        </is>
-      </c>
-      <c r="E189" s="5" t="inlineStr">
-        <is>
-          <t>Effort</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="7" t="n">
-        <v>188</v>
-      </c>
-      <c r="B190" s="8" t="n">
-        <v>46262</v>
-      </c>
-      <c r="C190" s="9" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-      <c r="D190" s="10" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E190" s="9" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="3" t="n">
-        <v>189</v>
-      </c>
-      <c r="B191" s="4" t="n">
-        <v>46263</v>
-      </c>
-      <c r="C191" s="5" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D191" s="6" t="inlineStr">
-        <is>
-          <t>2:4</t>
-        </is>
-      </c>
-      <c r="E191" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="7" t="n">
-        <v>190</v>
-      </c>
-      <c r="B192" s="8" t="n">
-        <v>46264</v>
-      </c>
-      <c r="C192" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D192" s="10" t="inlineStr">
-        <is>
-          <t>3:4</t>
-        </is>
-      </c>
-      <c r="E192" s="9" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="3" t="n">
-        <v>191</v>
-      </c>
-      <c r="B193" s="4" t="n">
-        <v>46265</v>
-      </c>
-      <c r="C193" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D193" s="6" t="inlineStr">
-        <is>
-          <t>2:4</t>
-        </is>
-      </c>
-      <c r="E193" s="5" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="7" t="n">
-        <v>192</v>
-      </c>
-      <c r="B194" s="8" t="n">
-        <v>46266</v>
-      </c>
-      <c r="C194" s="9" t="inlineStr">
-        <is>
-          <t>Mini</t>
-        </is>
-      </c>
-      <c r="D194" s="10" t="inlineStr">
-        <is>
-          <t>3:4</t>
-        </is>
-      </c>
-      <c r="E194" s="9" t="inlineStr">
-        <is>
-          <t>Rush</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="3" t="n">
-        <v>193</v>
-      </c>
-      <c r="B195" s="4" t="n">
-        <v>46267</v>
-      </c>
-      <c r="C195" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D195" s="6" t="inlineStr">
-        <is>
-          <t>3:4</t>
-        </is>
-      </c>
-      <c r="E195" s="5" t="inlineStr">
-        <is>
-          <t>Soulkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="7" t="n">
-        <v>194</v>
-      </c>
-      <c r="B196" s="8" t="n">
-        <v>46268</v>
-      </c>
-      <c r="C196" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D196" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E196" s="9" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="B197" s="4" t="n">
-        <v>46269</v>
-      </c>
-      <c r="C197" s="5" t="inlineStr">
-        <is>
-          <t>Rush</t>
-        </is>
-      </c>
-      <c r="D197" s="6" t="inlineStr">
-        <is>
-          <t>2:4</t>
-        </is>
-      </c>
-      <c r="E197" s="5" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="7" t="n">
-        <v>196</v>
-      </c>
-      <c r="B198" s="8" t="n">
-        <v>46271</v>
-      </c>
-      <c r="C198" s="9" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="D198" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E198" s="9" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="3" t="n">
-        <v>197</v>
-      </c>
-      <c r="B199" s="4" t="n">
-        <v>46272</v>
-      </c>
-      <c r="C199" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="D199" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E199" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="7" t="n">
-        <v>198</v>
-      </c>
-      <c r="B200" s="8" t="n">
-        <v>46273</v>
-      </c>
-      <c r="C200" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D200" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E200" s="9" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="3" t="n">
-        <v>199</v>
-      </c>
-      <c r="B201" s="4" t="n">
-        <v>46274</v>
-      </c>
-      <c r="C201" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="D201" s="6" t="inlineStr">
-        <is>
-          <t>4:0</t>
-        </is>
-      </c>
-      <c r="E201" s="5" t="inlineStr">
-        <is>
-          <t>Mini</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="B202" s="8" t="n">
-        <v>46275</v>
-      </c>
-      <c r="C202" s="9" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-      <c r="D202" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E202" s="9" t="inlineStr">
-        <is>
-          <t>Soulkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="3" t="n">
-        <v>201</v>
-      </c>
-      <c r="B203" s="4" t="n">
-        <v>46277</v>
-      </c>
-      <c r="C203" s="5" t="inlineStr">
-        <is>
-          <t>Sorry</t>
-        </is>
-      </c>
-      <c r="D203" s="6" t="inlineStr">
-        <is>
-          <t>4:0</t>
-        </is>
-      </c>
-      <c r="E203" s="5" t="inlineStr">
-        <is>
-          <t>Soulkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="7" t="n">
-        <v>202</v>
-      </c>
-      <c r="B204" s="8" t="n">
-        <v>46278</v>
-      </c>
-      <c r="C204" s="9" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-      <c r="D204" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E204" s="9" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" s="3" t="n">
-        <v>203</v>
-      </c>
-      <c r="B205" s="4" t="n">
-        <v>46279</v>
-      </c>
-      <c r="C205" s="5" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="D205" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E205" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" s="7" t="n">
-        <v>204</v>
-      </c>
-      <c r="B206" s="8" t="n">
-        <v>46280</v>
-      </c>
-      <c r="C206" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D206" s="10" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E206" s="9" t="inlineStr">
-        <is>
-          <t>Soma</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" s="3" t="n">
-        <v>205</v>
-      </c>
-      <c r="B207" s="4" t="n">
-        <v>46282</v>
-      </c>
-      <c r="C207" s="5" t="inlineStr">
-        <is>
-          <t>Rush</t>
-        </is>
-      </c>
-      <c r="D207" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E207" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="7" t="n">
-        <v>206</v>
-      </c>
-      <c r="B208" s="8" t="n">
-        <v>46283</v>
-      </c>
-      <c r="C208" s="9" t="inlineStr">
-        <is>
-          <t>Stork</t>
-        </is>
-      </c>
-      <c r="D208" s="10" t="inlineStr">
-        <is>
-          <t>4:0</t>
-        </is>
-      </c>
-      <c r="E208" s="9" t="inlineStr">
-        <is>
-          <t>迷糊</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" s="3" t="n">
-        <v>207</v>
-      </c>
-      <c r="B209" s="4" t="n">
-        <v>46284</v>
-      </c>
-      <c r="C209" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="D209" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="E209" s="5" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" s="7" t="n">
-        <v>208</v>
-      </c>
-      <c r="B210" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="C210" s="9" t="inlineStr">
-        <is>
-          <t>Sharp</t>
-        </is>
-      </c>
-      <c r="D210" s="10" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E210" s="9" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" s="3" t="n">
-        <v>209</v>
-      </c>
-      <c r="B211" s="4" t="n">
-        <v>46286</v>
-      </c>
-      <c r="C211" s="5" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="D211" s="6" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E211" s="5" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" s="7" t="n">
-        <v>210</v>
-      </c>
-      <c r="B212" s="8" t="n">
-        <v>46287</v>
-      </c>
-      <c r="C212" s="9" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="D212" s="10" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="E212" s="9" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" s="3" t="n">
-        <v>211</v>
-      </c>
-      <c r="B213" s="4" t="n">
-        <v>46288</v>
-      </c>
-      <c r="C213" s="5" t="inlineStr">
-        <is>
-          <t>Best</t>
-        </is>
-      </c>
-      <c r="D213" s="6" t="inlineStr">
-        <is>
-          <t>4:3</t>
-        </is>
-      </c>
-      <c r="E213" s="5" t="inlineStr">
-        <is>
-          <t>Sorry</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="7" t="n">
-        <v>212</v>
-      </c>
-      <c r="B214" s="8" t="n">
-        <v>46289</v>
-      </c>
-      <c r="C214" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D214" s="10" t="inlineStr">
-        <is>
-          <t>2:4</t>
-        </is>
-      </c>
-      <c r="E214" s="9" t="inlineStr">
-        <is>
-          <t>Soulkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" s="3" t="n">
-        <v>213</v>
-      </c>
-      <c r="B215" s="4" t="n">
-        <v>46290</v>
-      </c>
-      <c r="C215" s="5" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D215" s="6" t="inlineStr">
-        <is>
-          <t>0:4</t>
-        </is>
-      </c>
-      <c r="E215" s="5" t="inlineStr">
-        <is>
-          <t>JD</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:E215"/>
+  <autoFilter ref="A2:E141"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5488,7 +3786,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-01-01 至 2026-09-18，共 213 场「巅峰赛场」对局。</t>
+          <t>2026-01-01 至 2026-09-18，共 139 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-09-29（共 217 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$215</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$219</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E215"/>
+  <dimension ref="A1:E219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5439,8 +5439,100 @@
         </is>
       </c>
     </row>
+    <row r="216">
+      <c r="A216" s="7" t="n">
+        <v>214</v>
+      </c>
+      <c r="B216" s="8" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C216" s="9" t="inlineStr">
+        <is>
+          <t>Sorry</t>
+        </is>
+      </c>
+      <c r="D216" s="10" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E216" s="9" t="inlineStr">
+        <is>
+          <t>Soulkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="B217" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="C217" s="5" t="inlineStr">
+        <is>
+          <t>永镇</t>
+        </is>
+      </c>
+      <c r="D217" s="6" t="inlineStr">
+        <is>
+          <t>4:3</t>
+        </is>
+      </c>
+      <c r="E217" s="5" t="inlineStr">
+        <is>
+          <t>永康</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="7" t="n">
+        <v>216</v>
+      </c>
+      <c r="B218" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C218" s="9" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="D218" s="10" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E218" s="9" t="inlineStr">
+        <is>
+          <t>Mini</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="n">
+        <v>217</v>
+      </c>
+      <c r="B219" s="4" t="n">
+        <v>46294</v>
+      </c>
+      <c r="C219" s="5" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D219" s="6" t="inlineStr">
+        <is>
+          <t>4:3</t>
+        </is>
+      </c>
+      <c r="E219" s="5" t="inlineStr">
+        <is>
+          <t>Hero</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E215"/>
+  <autoFilter ref="A2:E219"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5488,7 +5580,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-01-01 至 2026-09-18，共 213 场「巅峰赛场」对局。</t>
+          <t>2026-01-01 至 2026-09-18，共 217 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-10-07（共 224 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="巅峰赛场战绩" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="巅峰赛场战绩" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$219</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$226</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E219"/>
+  <dimension ref="A1:E226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5531,8 +5531,169 @@
         </is>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" s="7" t="n">
+        <v>218</v>
+      </c>
+      <c r="B220" s="8" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C220" s="9" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="D220" s="10" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E220" s="9" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="n">
+        <v>219</v>
+      </c>
+      <c r="B221" s="4" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C221" s="5" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D221" s="6" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E221" s="5" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="B222" s="8" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C222" s="9" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D222" s="10" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
+      <c r="E222" s="9" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="3" t="n">
+        <v>221</v>
+      </c>
+      <c r="B223" s="4" t="n">
+        <v>46298</v>
+      </c>
+      <c r="C223" s="5" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D223" s="6" t="inlineStr">
+        <is>
+          <t>3:4</t>
+        </is>
+      </c>
+      <c r="E223" s="5" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="7" t="n">
+        <v>222</v>
+      </c>
+      <c r="B224" s="8" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C224" s="9" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+      <c r="D224" s="10" t="inlineStr">
+        <is>
+          <t>2:4</t>
+        </is>
+      </c>
+      <c r="E224" s="9" t="inlineStr">
+        <is>
+          <t>Sorry</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="n">
+        <v>223</v>
+      </c>
+      <c r="B225" s="4" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C225" s="5" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+      <c r="D225" s="6" t="inlineStr">
+        <is>
+          <t>2:4</t>
+        </is>
+      </c>
+      <c r="E225" s="5" t="inlineStr">
+        <is>
+          <t>Sorry</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="7" t="n">
+        <v>224</v>
+      </c>
+      <c r="B226" s="8" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C226" s="9" t="inlineStr">
+        <is>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="D226" s="10" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E226" s="9" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E219"/>
+  <autoFilter ref="A2:E226"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5580,7 +5741,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-01-01 至 2026-09-18，共 217 场「巅峰赛场」对局。</t>
+          <t>2026-01-01 至 2026-09-18，共 224 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-10-10（共 227 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$226</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$229</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E226"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5692,8 +5692,77 @@
         </is>
       </c>
     </row>
+    <row r="227">
+      <c r="A227" s="3" t="n">
+        <v>225</v>
+      </c>
+      <c r="B227" s="4" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C227" s="5" t="inlineStr">
+        <is>
+          <t>Snow</t>
+        </is>
+      </c>
+      <c r="D227" s="6" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
+      <c r="E227" s="5" t="inlineStr">
+        <is>
+          <t>Rush</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="7" t="n">
+        <v>226</v>
+      </c>
+      <c r="B228" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C228" s="9" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D228" s="10" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
+      <c r="E228" s="9" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="3" t="n">
+        <v>227</v>
+      </c>
+      <c r="B229" s="4" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C229" s="5" t="inlineStr">
+        <is>
+          <t>Mini</t>
+        </is>
+      </c>
+      <c r="D229" s="6" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E229" s="5" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E226"/>
+  <autoFilter ref="A2:E229"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5741,7 +5810,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-01-01 至 2026-09-18，共 224 场「巅峰赛场」对局。</t>
+          <t>2026-01-01 至 2026-09-18，共 227 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-10-13（共 228 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$229</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$230</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5761,8 +5761,31 @@
         </is>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" s="7" t="n">
+        <v>228</v>
+      </c>
+      <c r="B230" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C230" s="9" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D230" s="10" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="E230" s="9" t="inlineStr">
+        <is>
+          <t>Hero</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E229"/>
+  <autoFilter ref="A2:E230"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5776,7 +5799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5805,60 +5828,72 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>统计范围</t>
+          <t>人工补录</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-01-01 至 2026-09-18，共 227 场「巅峰赛场」对局。</t>
+          <t>其中 1 条因归档站收录滞后，按公众号原文人工补录（见 peak-arena-ledger/data/manual_records.json）；归档站补收录后会自动以解析结果为准。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>日期口径</t>
+          <t>统计范围</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>战报为次日发布，标题即「昨日战报」，故表中日期 = 战报发布日 − 1 天，即实际比赛日。</t>
+          <t>2026-01-05 至 2026-10-13，共 228 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>抓取范围</t>
+          <t>日期口径</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>该公众号 2025-12-01 至 2026-09-20 全部 277 篇推文，其中 196 篇含「巅峰赛场」条目。</t>
+          <t>战报为次日发布，标题即「昨日战报」，故表中日期 = 战报发布日 − 1 天，即实际比赛日。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>说明</t>
+          <t>抓取范围</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>同一日出现两行（如 bo7+bo3）时，为该日安排了两场巅峰赛场对局。</t>
+          <t>该公众号 2025-12 起的历史推文全量抓取，仅统计「华府卫视战报」中「巅峰赛场」条目的对局。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>抓取时间</t>
+          <t>说明</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>同一日出现两行（如 bo7+bo3）时，为该日安排了两场巅峰赛场对局。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>数据更新</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>由 peak-arena-ledger/daily_update.py 每日自动增量更新；具体变更见仓库提交记录。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-10-13（共 230 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$230</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$232</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E230"/>
+  <dimension ref="A1:E232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5766,26 +5766,72 @@
         <v>228</v>
       </c>
       <c r="B230" s="8" t="n">
+        <v>46306</v>
+      </c>
+      <c r="C230" s="9" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="D230" s="10" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E230" s="9" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="n">
+        <v>229</v>
+      </c>
+      <c r="B231" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C231" s="5" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D231" s="6" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="E231" s="5" t="inlineStr">
+        <is>
+          <t>JD</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="B232" s="8" t="n">
         <v>46308</v>
       </c>
-      <c r="C230" s="9" t="inlineStr">
-        <is>
-          <t>Bisu</t>
-        </is>
-      </c>
-      <c r="D230" s="10" t="inlineStr">
+      <c r="C232" s="9" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D232" s="10" t="inlineStr">
         <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="E230" s="9" t="inlineStr">
+      <c r="E232" s="9" t="inlineStr">
         <is>
           <t>Hero</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:E230"/>
+  <autoFilter ref="A2:E232"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5833,7 +5879,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>其中 1 条因归档站收录滞后，按公众号原文人工补录（见 peak-arena-ledger/data/manual_records.json）；归档站补收录后会自动以解析结果为准。</t>
+          <t>其中 3 条因归档站收录滞后，按公众号原文人工补录（见 peak-arena-ledger/data/manual_records.json）；归档站补收录后会自动以解析结果为准。</t>
         </is>
       </c>
     </row>
@@ -5845,7 +5891,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>2026-01-05 至 2026-10-13，共 228 场「巅峰赛场」对局。</t>
+          <t>2026-01-05 至 2026-10-13，共 230 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-10-16（共 232 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$232</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$234</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E232"/>
+  <dimension ref="A1:E234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5830,8 +5830,54 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" s="3" t="n">
+        <v>231</v>
+      </c>
+      <c r="B233" s="4" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C233" s="5" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+      <c r="D233" s="6" t="inlineStr">
+        <is>
+          <t>4:3</t>
+        </is>
+      </c>
+      <c r="E233" s="5" t="inlineStr">
+        <is>
+          <t>Sorry</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="7" t="n">
+        <v>232</v>
+      </c>
+      <c r="B234" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C234" s="9" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+      <c r="D234" s="10" t="inlineStr">
+        <is>
+          <t>3:4</t>
+        </is>
+      </c>
+      <c r="E234" s="9" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E232"/>
+  <autoFilter ref="A2:E234"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5891,7 +5937,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>2026-01-05 至 2026-10-13，共 230 场「巅峰赛场」对局。</t>
+          <t>2026-01-05 至 2026-10-16，共 232 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-10-19（共 235 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$234</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$237</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E234"/>
+  <dimension ref="A1:E237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5876,8 +5876,77 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" s="3" t="n">
+        <v>233</v>
+      </c>
+      <c r="B235" s="4" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C235" s="5" t="inlineStr">
+        <is>
+          <t>迷糊</t>
+        </is>
+      </c>
+      <c r="D235" s="6" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="E235" s="5" t="inlineStr">
+        <is>
+          <t>Stork</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="7" t="n">
+        <v>234</v>
+      </c>
+      <c r="B236" s="8" t="n">
+        <v>46313</v>
+      </c>
+      <c r="C236" s="9" t="inlineStr">
+        <is>
+          <t>Sorry</t>
+        </is>
+      </c>
+      <c r="D236" s="10" t="inlineStr">
+        <is>
+          <t>3:4</t>
+        </is>
+      </c>
+      <c r="E236" s="9" t="inlineStr">
+        <is>
+          <t>Soma</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="3" t="n">
+        <v>235</v>
+      </c>
+      <c r="B237" s="4" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C237" s="5" t="inlineStr">
+        <is>
+          <t>Soma</t>
+        </is>
+      </c>
+      <c r="D237" s="6" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
+      <c r="E237" s="5" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E234"/>
+  <autoFilter ref="A2:E237"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5937,7 +6006,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>2026-01-05 至 2026-10-16，共 232 场「巅峰赛场」对局。</t>
+          <t>2026-01-05 至 2026-10-19，共 235 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): 同步 2026-10-22（共 238 场）
</commit_message>
<xml_diff>
--- a/华府卫视巅峰赛场战绩_2026.xlsx
+++ b/华府卫视巅峰赛场战绩_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="数据说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'巅峰赛场战绩'!$A$2:$E$240</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E237"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5945,8 +5945,77 @@
         </is>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" s="7" t="n">
+        <v>236</v>
+      </c>
+      <c r="B238" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C238" s="9" t="inlineStr">
+        <is>
+          <t>Snow</t>
+        </is>
+      </c>
+      <c r="D238" s="10" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="E238" s="9" t="inlineStr">
+        <is>
+          <t>Soma</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="3" t="n">
+        <v>237</v>
+      </c>
+      <c r="B239" s="4" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C239" s="5" t="inlineStr">
+        <is>
+          <t>SPeed</t>
+        </is>
+      </c>
+      <c r="D239" s="6" t="inlineStr">
+        <is>
+          <t>4:3</t>
+        </is>
+      </c>
+      <c r="E239" s="5" t="inlineStr">
+        <is>
+          <t>JD</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="7" t="n">
+        <v>238</v>
+      </c>
+      <c r="B240" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C240" s="9" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="D240" s="10" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
+      <c r="E240" s="9" t="inlineStr">
+        <is>
+          <t>Bisu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:E237"/>
+  <autoFilter ref="A2:E240"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -6006,7 +6075,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>2026-01-05 至 2026-10-19，共 235 场「巅峰赛场」对局。</t>
+          <t>2026-01-05 至 2026-10-22，共 238 场「巅峰赛场」对局。</t>
         </is>
       </c>
     </row>

</xml_diff>